<commit_message>
Update sweep_results_hybrid_G1.xlsx with new analysis data
</commit_message>
<xml_diff>
--- a/Data_Analysis/Sensitivity analysis/Hybrid/sweep_results_hybrid_G1.xlsx
+++ b/Data_Analysis/Sensitivity analysis/Hybrid/sweep_results_hybrid_G1.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="3626" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="3766" uniqueCount="14">
   <si>
     <t>RUN_ID</t>
   </si>
@@ -100,7 +100,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N260"/>
+  <dimension ref="A1:N270"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.5546875" customWidth="true"/>
@@ -11559,6 +11559,446 @@
         <v>5.2658233457694905</v>
       </c>
     </row>
+    <row r="261">
+      <c r="A261" s="0">
+        <v>101</v>
+      </c>
+      <c r="B261" s="0">
+        <v>260</v>
+      </c>
+      <c r="C261" s="0">
+        <v>101</v>
+      </c>
+      <c r="D261" s="0">
+        <v>93.696156067053522</v>
+      </c>
+      <c r="E261" s="0">
+        <v>477.73500000000001</v>
+      </c>
+      <c r="F261" s="0">
+        <v>154.16829868763406</v>
+      </c>
+      <c r="G261" s="0">
+        <v>5425.7414909559302</v>
+      </c>
+      <c r="H261" s="0">
+        <v>-1332.1129555774955</v>
+      </c>
+      <c r="I261" s="0">
+        <v>5.8150000000000004</v>
+      </c>
+      <c r="J261" s="0">
+        <v>16.82</v>
+      </c>
+      <c r="K261" s="0">
+        <v>2.6399999999999997</v>
+      </c>
+      <c r="L261" s="0">
+        <v>3.71</v>
+      </c>
+      <c r="M261" s="0">
+        <v>288.5495800015193</v>
+      </c>
+      <c r="N261" s="0">
+        <v>5.2658233457694905</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="0">
+        <v>101</v>
+      </c>
+      <c r="B262" s="0">
+        <v>261</v>
+      </c>
+      <c r="C262" s="0">
+        <v>101</v>
+      </c>
+      <c r="D262" s="0">
+        <v>93.696156067053522</v>
+      </c>
+      <c r="E262" s="0">
+        <v>477.73500000000001</v>
+      </c>
+      <c r="F262" s="0">
+        <v>154.16829868763406</v>
+      </c>
+      <c r="G262" s="0">
+        <v>5425.7414909559302</v>
+      </c>
+      <c r="H262" s="0">
+        <v>-1332.1129555774955</v>
+      </c>
+      <c r="I262" s="0">
+        <v>5.8150000000000004</v>
+      </c>
+      <c r="J262" s="0">
+        <v>16.82</v>
+      </c>
+      <c r="K262" s="0">
+        <v>2.6399999999999997</v>
+      </c>
+      <c r="L262" s="0">
+        <v>3.71</v>
+      </c>
+      <c r="M262" s="0">
+        <v>288.5495800015193</v>
+      </c>
+      <c r="N262" s="0">
+        <v>5.2658233457694905</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="0">
+        <v>101</v>
+      </c>
+      <c r="B263" s="0">
+        <v>262</v>
+      </c>
+      <c r="C263" s="0">
+        <v>101</v>
+      </c>
+      <c r="D263" s="0">
+        <v>93.696156067053522</v>
+      </c>
+      <c r="E263" s="0">
+        <v>477.73500000000001</v>
+      </c>
+      <c r="F263" s="0">
+        <v>154.16829868763406</v>
+      </c>
+      <c r="G263" s="0">
+        <v>5425.7414909559302</v>
+      </c>
+      <c r="H263" s="0">
+        <v>-1332.1129555774955</v>
+      </c>
+      <c r="I263" s="0">
+        <v>5.8150000000000004</v>
+      </c>
+      <c r="J263" s="0">
+        <v>16.82</v>
+      </c>
+      <c r="K263" s="0">
+        <v>2.6399999999999997</v>
+      </c>
+      <c r="L263" s="0">
+        <v>3.71</v>
+      </c>
+      <c r="M263" s="0">
+        <v>288.5495800015193</v>
+      </c>
+      <c r="N263" s="0">
+        <v>5.2658233457694905</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="0">
+        <v>101</v>
+      </c>
+      <c r="B264" s="0">
+        <v>263</v>
+      </c>
+      <c r="C264" s="0">
+        <v>101</v>
+      </c>
+      <c r="D264" s="0">
+        <v>93.696156067053522</v>
+      </c>
+      <c r="E264" s="0">
+        <v>477.73500000000001</v>
+      </c>
+      <c r="F264" s="0">
+        <v>154.16829868763406</v>
+      </c>
+      <c r="G264" s="0">
+        <v>5425.7414909559302</v>
+      </c>
+      <c r="H264" s="0">
+        <v>-1332.1129555774955</v>
+      </c>
+      <c r="I264" s="0">
+        <v>5.8150000000000004</v>
+      </c>
+      <c r="J264" s="0">
+        <v>16.82</v>
+      </c>
+      <c r="K264" s="0">
+        <v>2.6399999999999997</v>
+      </c>
+      <c r="L264" s="0">
+        <v>3.71</v>
+      </c>
+      <c r="M264" s="0">
+        <v>288.5495800015193</v>
+      </c>
+      <c r="N264" s="0">
+        <v>5.2658233457694905</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="0">
+        <v>101</v>
+      </c>
+      <c r="B265" s="0">
+        <v>264</v>
+      </c>
+      <c r="C265" s="0">
+        <v>101</v>
+      </c>
+      <c r="D265" s="0">
+        <v>93.696156067053522</v>
+      </c>
+      <c r="E265" s="0">
+        <v>477.73500000000001</v>
+      </c>
+      <c r="F265" s="0">
+        <v>154.16829868763406</v>
+      </c>
+      <c r="G265" s="0">
+        <v>5425.7414909559302</v>
+      </c>
+      <c r="H265" s="0">
+        <v>-1332.1129555774955</v>
+      </c>
+      <c r="I265" s="0">
+        <v>5.8150000000000004</v>
+      </c>
+      <c r="J265" s="0">
+        <v>16.82</v>
+      </c>
+      <c r="K265" s="0">
+        <v>2.6399999999999997</v>
+      </c>
+      <c r="L265" s="0">
+        <v>3.71</v>
+      </c>
+      <c r="M265" s="0">
+        <v>288.5495800015193</v>
+      </c>
+      <c r="N265" s="0">
+        <v>5.2658233457694905</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="0">
+        <v>101</v>
+      </c>
+      <c r="B266" s="0">
+        <v>265</v>
+      </c>
+      <c r="C266" s="0">
+        <v>101</v>
+      </c>
+      <c r="D266" s="0">
+        <v>93.672505857068415</v>
+      </c>
+      <c r="E266" s="0">
+        <v>474.69</v>
+      </c>
+      <c r="F266" s="0">
+        <v>155.15724404039872</v>
+      </c>
+      <c r="G266" s="0">
+        <v>5592.5244255291755</v>
+      </c>
+      <c r="H266" s="0">
+        <v>-1426.7200279218582</v>
+      </c>
+      <c r="I266" s="0">
+        <v>5.7999999999999998</v>
+      </c>
+      <c r="J266" s="0">
+        <v>16.215</v>
+      </c>
+      <c r="K266" s="0">
+        <v>2.5450000000000008</v>
+      </c>
+      <c r="L266" s="0">
+        <v>3.6150000000000007</v>
+      </c>
+      <c r="M266" s="0">
+        <v>293.08003750361371</v>
+      </c>
+      <c r="N266" s="0">
+        <v>5.2658384210157783</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="0">
+        <v>101</v>
+      </c>
+      <c r="B267" s="0">
+        <v>266</v>
+      </c>
+      <c r="C267" s="0">
+        <v>101</v>
+      </c>
+      <c r="D267" s="0">
+        <v>93.672505857068415</v>
+      </c>
+      <c r="E267" s="0">
+        <v>474.69</v>
+      </c>
+      <c r="F267" s="0">
+        <v>155.15724404039872</v>
+      </c>
+      <c r="G267" s="0">
+        <v>5592.5244255291755</v>
+      </c>
+      <c r="H267" s="0">
+        <v>-1426.7200279218582</v>
+      </c>
+      <c r="I267" s="0">
+        <v>5.7999999999999998</v>
+      </c>
+      <c r="J267" s="0">
+        <v>16.215</v>
+      </c>
+      <c r="K267" s="0">
+        <v>2.5450000000000008</v>
+      </c>
+      <c r="L267" s="0">
+        <v>3.6150000000000007</v>
+      </c>
+      <c r="M267" s="0">
+        <v>293.08003750361371</v>
+      </c>
+      <c r="N267" s="0">
+        <v>5.2658384210157783</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="0">
+        <v>101</v>
+      </c>
+      <c r="B268" s="0">
+        <v>267</v>
+      </c>
+      <c r="C268" s="0">
+        <v>101</v>
+      </c>
+      <c r="D268" s="0">
+        <v>93.672505857068415</v>
+      </c>
+      <c r="E268" s="0">
+        <v>474.69</v>
+      </c>
+      <c r="F268" s="0">
+        <v>155.15724404039872</v>
+      </c>
+      <c r="G268" s="0">
+        <v>5592.5244255291755</v>
+      </c>
+      <c r="H268" s="0">
+        <v>-1426.7200279218582</v>
+      </c>
+      <c r="I268" s="0">
+        <v>5.7999999999999998</v>
+      </c>
+      <c r="J268" s="0">
+        <v>16.215</v>
+      </c>
+      <c r="K268" s="0">
+        <v>2.5450000000000008</v>
+      </c>
+      <c r="L268" s="0">
+        <v>3.6150000000000007</v>
+      </c>
+      <c r="M268" s="0">
+        <v>293.08003750361371</v>
+      </c>
+      <c r="N268" s="0">
+        <v>5.2658384210157783</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="0">
+        <v>101</v>
+      </c>
+      <c r="B269" s="0">
+        <v>268</v>
+      </c>
+      <c r="C269" s="0">
+        <v>101</v>
+      </c>
+      <c r="D269" s="0">
+        <v>93.672505857068415</v>
+      </c>
+      <c r="E269" s="0">
+        <v>474.69</v>
+      </c>
+      <c r="F269" s="0">
+        <v>155.15724404039872</v>
+      </c>
+      <c r="G269" s="0">
+        <v>5592.5244255291755</v>
+      </c>
+      <c r="H269" s="0">
+        <v>-1426.7200279218582</v>
+      </c>
+      <c r="I269" s="0">
+        <v>5.7999999999999998</v>
+      </c>
+      <c r="J269" s="0">
+        <v>16.215</v>
+      </c>
+      <c r="K269" s="0">
+        <v>2.5450000000000008</v>
+      </c>
+      <c r="L269" s="0">
+        <v>3.6150000000000007</v>
+      </c>
+      <c r="M269" s="0">
+        <v>293.08003750361371</v>
+      </c>
+      <c r="N269" s="0">
+        <v>5.2658384210157783</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="0">
+        <v>101</v>
+      </c>
+      <c r="B270" s="0">
+        <v>269</v>
+      </c>
+      <c r="C270" s="0">
+        <v>101</v>
+      </c>
+      <c r="D270" s="0">
+        <v>93.672505857068415</v>
+      </c>
+      <c r="E270" s="0">
+        <v>474.69</v>
+      </c>
+      <c r="F270" s="0">
+        <v>155.15724404039872</v>
+      </c>
+      <c r="G270" s="0">
+        <v>5592.5244255291755</v>
+      </c>
+      <c r="H270" s="0">
+        <v>-1426.7200279218582</v>
+      </c>
+      <c r="I270" s="0">
+        <v>5.7999999999999998</v>
+      </c>
+      <c r="J270" s="0">
+        <v>16.215</v>
+      </c>
+      <c r="K270" s="0">
+        <v>2.5450000000000008</v>
+      </c>
+      <c r="L270" s="0">
+        <v>3.6150000000000007</v>
+      </c>
+      <c r="M270" s="0">
+        <v>293.08003750361371</v>
+      </c>
+      <c r="N270" s="0">
+        <v>5.2658384210157783</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update sweep_results_hybrid_G1.xlsx with revised analysis results
</commit_message>
<xml_diff>
--- a/Data_Analysis/Sensitivity analysis/Hybrid/sweep_results_hybrid_G1.xlsx
+++ b/Data_Analysis/Sensitivity analysis/Hybrid/sweep_results_hybrid_G1.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="3766" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="3878" uniqueCount="14">
   <si>
     <t>RUN_ID</t>
   </si>
@@ -100,7 +100,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N270"/>
+  <dimension ref="A1:N278"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.5546875" customWidth="true"/>
@@ -11999,6 +11999,358 @@
         <v>5.2658384210157783</v>
       </c>
     </row>
+    <row r="271">
+      <c r="A271" s="0">
+        <v>101</v>
+      </c>
+      <c r="B271" s="0">
+        <v>270</v>
+      </c>
+      <c r="C271" s="0">
+        <v>101</v>
+      </c>
+      <c r="D271" s="0">
+        <v>93.672505857068415</v>
+      </c>
+      <c r="E271" s="0">
+        <v>474.69</v>
+      </c>
+      <c r="F271" s="0">
+        <v>155.15724404039872</v>
+      </c>
+      <c r="G271" s="0">
+        <v>5592.5244255291755</v>
+      </c>
+      <c r="H271" s="0">
+        <v>-1426.7200279218582</v>
+      </c>
+      <c r="I271" s="0">
+        <v>5.7999999999999998</v>
+      </c>
+      <c r="J271" s="0">
+        <v>16.215</v>
+      </c>
+      <c r="K271" s="0">
+        <v>2.5450000000000008</v>
+      </c>
+      <c r="L271" s="0">
+        <v>3.6150000000000007</v>
+      </c>
+      <c r="M271" s="0">
+        <v>293.08003750361371</v>
+      </c>
+      <c r="N271" s="0">
+        <v>5.2658384210157783</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="0">
+        <v>101</v>
+      </c>
+      <c r="B272" s="0">
+        <v>271</v>
+      </c>
+      <c r="C272" s="0">
+        <v>101</v>
+      </c>
+      <c r="D272" s="0">
+        <v>93.672505857068415</v>
+      </c>
+      <c r="E272" s="0">
+        <v>474.69</v>
+      </c>
+      <c r="F272" s="0">
+        <v>155.15724404039872</v>
+      </c>
+      <c r="G272" s="0">
+        <v>5592.5244255291755</v>
+      </c>
+      <c r="H272" s="0">
+        <v>-1426.7200279218582</v>
+      </c>
+      <c r="I272" s="0">
+        <v>5.7999999999999998</v>
+      </c>
+      <c r="J272" s="0">
+        <v>16.215</v>
+      </c>
+      <c r="K272" s="0">
+        <v>2.5450000000000008</v>
+      </c>
+      <c r="L272" s="0">
+        <v>3.6150000000000007</v>
+      </c>
+      <c r="M272" s="0">
+        <v>293.08003750361371</v>
+      </c>
+      <c r="N272" s="0">
+        <v>5.2658384210157783</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="0">
+        <v>101</v>
+      </c>
+      <c r="B273" s="0">
+        <v>272</v>
+      </c>
+      <c r="C273" s="0">
+        <v>101</v>
+      </c>
+      <c r="D273" s="0">
+        <v>93.672505857068415</v>
+      </c>
+      <c r="E273" s="0">
+        <v>474.69</v>
+      </c>
+      <c r="F273" s="0">
+        <v>155.15724404039872</v>
+      </c>
+      <c r="G273" s="0">
+        <v>5592.5244255291755</v>
+      </c>
+      <c r="H273" s="0">
+        <v>-1426.7200279218582</v>
+      </c>
+      <c r="I273" s="0">
+        <v>5.7999999999999998</v>
+      </c>
+      <c r="J273" s="0">
+        <v>16.215</v>
+      </c>
+      <c r="K273" s="0">
+        <v>2.5450000000000008</v>
+      </c>
+      <c r="L273" s="0">
+        <v>3.6150000000000007</v>
+      </c>
+      <c r="M273" s="0">
+        <v>293.08003750361371</v>
+      </c>
+      <c r="N273" s="0">
+        <v>5.2658384210157783</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="0">
+        <v>101</v>
+      </c>
+      <c r="B274" s="0">
+        <v>273</v>
+      </c>
+      <c r="C274" s="0">
+        <v>101</v>
+      </c>
+      <c r="D274" s="0">
+        <v>93.647623318955482</v>
+      </c>
+      <c r="E274" s="0">
+        <v>472.05500000000001</v>
+      </c>
+      <c r="F274" s="0">
+        <v>156.02332815781395</v>
+      </c>
+      <c r="G274" s="0">
+        <v>5762.8977758503142</v>
+      </c>
+      <c r="H274" s="0">
+        <v>-1521.1592339581434</v>
+      </c>
+      <c r="I274" s="0">
+        <v>5.7949999999999999</v>
+      </c>
+      <c r="J274" s="0">
+        <v>15.695</v>
+      </c>
+      <c r="K274" s="0">
+        <v>2.4799999999999995</v>
+      </c>
+      <c r="L274" s="0">
+        <v>3.5499999999999998</v>
+      </c>
+      <c r="M274" s="0">
+        <v>297.4785662356436</v>
+      </c>
+      <c r="N274" s="0">
+        <v>5.2658524197876817</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="0">
+        <v>101</v>
+      </c>
+      <c r="B275" s="0">
+        <v>274</v>
+      </c>
+      <c r="C275" s="0">
+        <v>101</v>
+      </c>
+      <c r="D275" s="0">
+        <v>93.647623318955482</v>
+      </c>
+      <c r="E275" s="0">
+        <v>472.05500000000001</v>
+      </c>
+      <c r="F275" s="0">
+        <v>156.02332815781395</v>
+      </c>
+      <c r="G275" s="0">
+        <v>5762.8977758503142</v>
+      </c>
+      <c r="H275" s="0">
+        <v>-1521.1592339581434</v>
+      </c>
+      <c r="I275" s="0">
+        <v>5.7949999999999999</v>
+      </c>
+      <c r="J275" s="0">
+        <v>15.695</v>
+      </c>
+      <c r="K275" s="0">
+        <v>2.4799999999999995</v>
+      </c>
+      <c r="L275" s="0">
+        <v>3.5499999999999998</v>
+      </c>
+      <c r="M275" s="0">
+        <v>297.4785662356436</v>
+      </c>
+      <c r="N275" s="0">
+        <v>5.2658524197876817</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="0">
+        <v>101</v>
+      </c>
+      <c r="B276" s="0">
+        <v>275</v>
+      </c>
+      <c r="C276" s="0">
+        <v>101</v>
+      </c>
+      <c r="D276" s="0">
+        <v>93.647623318955482</v>
+      </c>
+      <c r="E276" s="0">
+        <v>472.05500000000001</v>
+      </c>
+      <c r="F276" s="0">
+        <v>156.02332815781395</v>
+      </c>
+      <c r="G276" s="0">
+        <v>5762.8977758503142</v>
+      </c>
+      <c r="H276" s="0">
+        <v>-1521.1592339581434</v>
+      </c>
+      <c r="I276" s="0">
+        <v>5.7949999999999999</v>
+      </c>
+      <c r="J276" s="0">
+        <v>15.695</v>
+      </c>
+      <c r="K276" s="0">
+        <v>2.4799999999999995</v>
+      </c>
+      <c r="L276" s="0">
+        <v>3.5499999999999998</v>
+      </c>
+      <c r="M276" s="0">
+        <v>297.4785662356436</v>
+      </c>
+      <c r="N276" s="0">
+        <v>5.2658524197876817</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="0">
+        <v>101</v>
+      </c>
+      <c r="B277" s="0">
+        <v>276</v>
+      </c>
+      <c r="C277" s="0">
+        <v>101</v>
+      </c>
+      <c r="D277" s="0">
+        <v>93.647623318955482</v>
+      </c>
+      <c r="E277" s="0">
+        <v>472.05500000000001</v>
+      </c>
+      <c r="F277" s="0">
+        <v>156.02332815781395</v>
+      </c>
+      <c r="G277" s="0">
+        <v>5762.8977758503142</v>
+      </c>
+      <c r="H277" s="0">
+        <v>-1521.1592339581434</v>
+      </c>
+      <c r="I277" s="0">
+        <v>5.7949999999999999</v>
+      </c>
+      <c r="J277" s="0">
+        <v>15.695</v>
+      </c>
+      <c r="K277" s="0">
+        <v>2.4799999999999995</v>
+      </c>
+      <c r="L277" s="0">
+        <v>3.5499999999999998</v>
+      </c>
+      <c r="M277" s="0">
+        <v>297.4785662356436</v>
+      </c>
+      <c r="N277" s="0">
+        <v>5.2658524197876817</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="0">
+        <v>101</v>
+      </c>
+      <c r="B278" s="0">
+        <v>277</v>
+      </c>
+      <c r="C278" s="0">
+        <v>101</v>
+      </c>
+      <c r="D278" s="0">
+        <v>93.647623318955482</v>
+      </c>
+      <c r="E278" s="0">
+        <v>472.05500000000001</v>
+      </c>
+      <c r="F278" s="0">
+        <v>156.02332815781395</v>
+      </c>
+      <c r="G278" s="0">
+        <v>5762.8977758503142</v>
+      </c>
+      <c r="H278" s="0">
+        <v>-1521.1592339581434</v>
+      </c>
+      <c r="I278" s="0">
+        <v>5.7949999999999999</v>
+      </c>
+      <c r="J278" s="0">
+        <v>15.695</v>
+      </c>
+      <c r="K278" s="0">
+        <v>2.4799999999999995</v>
+      </c>
+      <c r="L278" s="0">
+        <v>3.5499999999999998</v>
+      </c>
+      <c r="M278" s="0">
+        <v>297.4785662356436</v>
+      </c>
+      <c r="N278" s="0">
+        <v>5.2658524197876817</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Enhance sensitivity pipeline with SLURM array support and chunked output handling
</commit_message>
<xml_diff>
--- a/Data_Analysis/Sensitivity analysis/Hybrid/sweep_results_hybrid_G1.xlsx
+++ b/Data_Analysis/Sensitivity analysis/Hybrid/sweep_results_hybrid_G1.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="3878" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="7434" uniqueCount="14">
   <si>
     <t>RUN_ID</t>
   </si>
@@ -100,23 +100,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N278"/>
+  <dimension ref="A1:N287"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.5546875" customWidth="true"/>
-    <col min="2" max="2" width="14.21875" customWidth="true"/>
-    <col min="3" max="3" width="12.77734375" customWidth="true"/>
-    <col min="4" max="4" width="11.5546875" customWidth="true"/>
-    <col min="5" max="5" width="8.88671875" customWidth="true"/>
-    <col min="6" max="6" width="14.77734375" customWidth="true"/>
-    <col min="7" max="7" width="19.109375" customWidth="true"/>
-    <col min="8" max="8" width="20.6640625" customWidth="true"/>
-    <col min="9" max="9" width="16.21875" customWidth="true"/>
-    <col min="10" max="10" width="16.21875" customWidth="true"/>
-    <col min="11" max="11" width="17.21875" customWidth="true"/>
-    <col min="12" max="12" width="17.21875" customWidth="true"/>
-    <col min="13" max="13" width="13" customWidth="true"/>
-    <col min="14" max="14" width="17.33203125" customWidth="true"/>
+    <col min="1" max="1" width="7.85546875" customWidth="true"/>
+    <col min="2" max="2" width="14.85546875" customWidth="true"/>
+    <col min="3" max="3" width="13.28515625" customWidth="true"/>
+    <col min="4" max="4" width="11.7109375" customWidth="true"/>
+    <col min="5" max="5" width="9.5703125" customWidth="true"/>
+    <col min="6" max="6" width="16.140625" customWidth="true"/>
+    <col min="7" max="7" width="20.85546875" customWidth="true"/>
+    <col min="8" max="8" width="22.5703125" customWidth="true"/>
+    <col min="9" max="9" width="17" customWidth="true"/>
+    <col min="10" max="10" width="17" customWidth="true"/>
+    <col min="11" max="11" width="18" customWidth="true"/>
+    <col min="12" max="12" width="18" customWidth="true"/>
+    <col min="13" max="13" width="14.140625" customWidth="true"/>
+    <col min="14" max="14" width="18.28515625" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -12351,6 +12351,402 @@
         <v>5.2658524197876817</v>
       </c>
     </row>
+    <row r="279">
+      <c r="A279" s="0">
+        <v>101</v>
+      </c>
+      <c r="B279" s="0">
+        <v>278</v>
+      </c>
+      <c r="C279" s="0">
+        <v>101</v>
+      </c>
+      <c r="D279" s="0">
+        <v>93.647623318955482</v>
+      </c>
+      <c r="E279" s="0">
+        <v>472.05500000000001</v>
+      </c>
+      <c r="F279" s="0">
+        <v>156.02332815781395</v>
+      </c>
+      <c r="G279" s="0">
+        <v>5762.8977758503142</v>
+      </c>
+      <c r="H279" s="0">
+        <v>-1521.1592339581434</v>
+      </c>
+      <c r="I279" s="0">
+        <v>5.7949999999999999</v>
+      </c>
+      <c r="J279" s="0">
+        <v>15.695</v>
+      </c>
+      <c r="K279" s="0">
+        <v>2.4799999999999995</v>
+      </c>
+      <c r="L279" s="0">
+        <v>3.5499999999999998</v>
+      </c>
+      <c r="M279" s="0">
+        <v>297.4785662356436</v>
+      </c>
+      <c r="N279" s="0">
+        <v>5.2658524197876817</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="0">
+        <v>101</v>
+      </c>
+      <c r="B280" s="0">
+        <v>279</v>
+      </c>
+      <c r="C280" s="0">
+        <v>101</v>
+      </c>
+      <c r="D280" s="0">
+        <v>93.647623318955482</v>
+      </c>
+      <c r="E280" s="0">
+        <v>472.05500000000001</v>
+      </c>
+      <c r="F280" s="0">
+        <v>156.02332815781395</v>
+      </c>
+      <c r="G280" s="0">
+        <v>5762.8977758503142</v>
+      </c>
+      <c r="H280" s="0">
+        <v>-1521.1592339581434</v>
+      </c>
+      <c r="I280" s="0">
+        <v>5.7949999999999999</v>
+      </c>
+      <c r="J280" s="0">
+        <v>15.695</v>
+      </c>
+      <c r="K280" s="0">
+        <v>2.4799999999999995</v>
+      </c>
+      <c r="L280" s="0">
+        <v>3.5499999999999998</v>
+      </c>
+      <c r="M280" s="0">
+        <v>297.4785662356436</v>
+      </c>
+      <c r="N280" s="0">
+        <v>5.2658524197876817</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="0">
+        <v>101</v>
+      </c>
+      <c r="B281" s="0">
+        <v>280</v>
+      </c>
+      <c r="C281" s="0">
+        <v>101</v>
+      </c>
+      <c r="D281" s="0">
+        <v>93.647623318955482</v>
+      </c>
+      <c r="E281" s="0">
+        <v>472.05500000000001</v>
+      </c>
+      <c r="F281" s="0">
+        <v>156.02332815781395</v>
+      </c>
+      <c r="G281" s="0">
+        <v>5762.8977758503142</v>
+      </c>
+      <c r="H281" s="0">
+        <v>-1521.1592339581434</v>
+      </c>
+      <c r="I281" s="0">
+        <v>5.7949999999999999</v>
+      </c>
+      <c r="J281" s="0">
+        <v>15.695</v>
+      </c>
+      <c r="K281" s="0">
+        <v>2.4799999999999995</v>
+      </c>
+      <c r="L281" s="0">
+        <v>3.5499999999999998</v>
+      </c>
+      <c r="M281" s="0">
+        <v>297.4785662356436</v>
+      </c>
+      <c r="N281" s="0">
+        <v>5.2658524197876817</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="0">
+        <v>103</v>
+      </c>
+      <c r="B282" s="0">
+        <v>281</v>
+      </c>
+      <c r="C282" s="0">
+        <v>103</v>
+      </c>
+      <c r="D282" s="0">
+        <v>94.211483600200324</v>
+      </c>
+      <c r="E282" s="0">
+        <v>473.76499999999999</v>
+      </c>
+      <c r="F282" s="0">
+        <v>155.46017999121267</v>
+      </c>
+      <c r="G282" s="0">
+        <v>3350.4679441746439</v>
+      </c>
+      <c r="H282" s="0">
+        <v>-867.06386050300739</v>
+      </c>
+      <c r="I282" s="0">
+        <v>5.8049999999999997</v>
+      </c>
+      <c r="J282" s="0">
+        <v>15.9</v>
+      </c>
+      <c r="K282" s="0">
+        <v>2.5949999999999998</v>
+      </c>
+      <c r="L282" s="0">
+        <v>3.6600000000000001</v>
+      </c>
+      <c r="M282" s="0">
+        <v>300.02869171301012</v>
+      </c>
+      <c r="N282" s="0">
+        <v>5.2712183117953497</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="0">
+        <v>103</v>
+      </c>
+      <c r="B283" s="0">
+        <v>282</v>
+      </c>
+      <c r="C283" s="0">
+        <v>103</v>
+      </c>
+      <c r="D283" s="0">
+        <v>94.211483600200324</v>
+      </c>
+      <c r="E283" s="0">
+        <v>473.76499999999999</v>
+      </c>
+      <c r="F283" s="0">
+        <v>155.46017999121267</v>
+      </c>
+      <c r="G283" s="0">
+        <v>3350.4679441746439</v>
+      </c>
+      <c r="H283" s="0">
+        <v>-867.06386050300739</v>
+      </c>
+      <c r="I283" s="0">
+        <v>5.8049999999999997</v>
+      </c>
+      <c r="J283" s="0">
+        <v>15.9</v>
+      </c>
+      <c r="K283" s="0">
+        <v>2.5949999999999998</v>
+      </c>
+      <c r="L283" s="0">
+        <v>3.6600000000000001</v>
+      </c>
+      <c r="M283" s="0">
+        <v>300.02869171301012</v>
+      </c>
+      <c r="N283" s="0">
+        <v>5.2712183117953497</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="0">
+        <v>103</v>
+      </c>
+      <c r="B284" s="0">
+        <v>283</v>
+      </c>
+      <c r="C284" s="0">
+        <v>103</v>
+      </c>
+      <c r="D284" s="0">
+        <v>94.211483600200324</v>
+      </c>
+      <c r="E284" s="0">
+        <v>473.76499999999999</v>
+      </c>
+      <c r="F284" s="0">
+        <v>155.46017999121267</v>
+      </c>
+      <c r="G284" s="0">
+        <v>3350.4679441746439</v>
+      </c>
+      <c r="H284" s="0">
+        <v>-867.06386050300739</v>
+      </c>
+      <c r="I284" s="0">
+        <v>5.8049999999999997</v>
+      </c>
+      <c r="J284" s="0">
+        <v>15.9</v>
+      </c>
+      <c r="K284" s="0">
+        <v>2.5949999999999998</v>
+      </c>
+      <c r="L284" s="0">
+        <v>3.6600000000000001</v>
+      </c>
+      <c r="M284" s="0">
+        <v>300.02869171301012</v>
+      </c>
+      <c r="N284" s="0">
+        <v>5.2712183117953497</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="0">
+        <v>103</v>
+      </c>
+      <c r="B285" s="0">
+        <v>284</v>
+      </c>
+      <c r="C285" s="0">
+        <v>103</v>
+      </c>
+      <c r="D285" s="0">
+        <v>94.211483600200324</v>
+      </c>
+      <c r="E285" s="0">
+        <v>473.76499999999999</v>
+      </c>
+      <c r="F285" s="0">
+        <v>155.46017999121267</v>
+      </c>
+      <c r="G285" s="0">
+        <v>3350.4679441746439</v>
+      </c>
+      <c r="H285" s="0">
+        <v>-867.06386050300739</v>
+      </c>
+      <c r="I285" s="0">
+        <v>5.8049999999999997</v>
+      </c>
+      <c r="J285" s="0">
+        <v>15.9</v>
+      </c>
+      <c r="K285" s="0">
+        <v>2.5949999999999998</v>
+      </c>
+      <c r="L285" s="0">
+        <v>3.6600000000000001</v>
+      </c>
+      <c r="M285" s="0">
+        <v>300.02869171301012</v>
+      </c>
+      <c r="N285" s="0">
+        <v>5.2712183117953497</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="0">
+        <v>103</v>
+      </c>
+      <c r="B286" s="0">
+        <v>285</v>
+      </c>
+      <c r="C286" s="0">
+        <v>103</v>
+      </c>
+      <c r="D286" s="0">
+        <v>94.211483600200324</v>
+      </c>
+      <c r="E286" s="0">
+        <v>473.76499999999999</v>
+      </c>
+      <c r="F286" s="0">
+        <v>155.46017999121267</v>
+      </c>
+      <c r="G286" s="0">
+        <v>3350.4679441746439</v>
+      </c>
+      <c r="H286" s="0">
+        <v>-867.06386050300739</v>
+      </c>
+      <c r="I286" s="0">
+        <v>5.8049999999999997</v>
+      </c>
+      <c r="J286" s="0">
+        <v>15.9</v>
+      </c>
+      <c r="K286" s="0">
+        <v>2.5949999999999998</v>
+      </c>
+      <c r="L286" s="0">
+        <v>3.6600000000000001</v>
+      </c>
+      <c r="M286" s="0">
+        <v>300.02869171301012</v>
+      </c>
+      <c r="N286" s="0">
+        <v>5.2712183117953497</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="0">
+        <v>103</v>
+      </c>
+      <c r="B287" s="0">
+        <v>286</v>
+      </c>
+      <c r="C287" s="0">
+        <v>103</v>
+      </c>
+      <c r="D287" s="0">
+        <v>94.211483600200324</v>
+      </c>
+      <c r="E287" s="0">
+        <v>473.76499999999999</v>
+      </c>
+      <c r="F287" s="0">
+        <v>155.46017999121267</v>
+      </c>
+      <c r="G287" s="0">
+        <v>3350.4679441746439</v>
+      </c>
+      <c r="H287" s="0">
+        <v>-867.06386050300739</v>
+      </c>
+      <c r="I287" s="0">
+        <v>5.8049999999999997</v>
+      </c>
+      <c r="J287" s="0">
+        <v>15.9</v>
+      </c>
+      <c r="K287" s="0">
+        <v>2.5949999999999998</v>
+      </c>
+      <c r="L287" s="0">
+        <v>3.6600000000000001</v>
+      </c>
+      <c r="M287" s="0">
+        <v>300.02869171301012</v>
+      </c>
+      <c r="N287" s="0">
+        <v>5.2712183117953497</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>